<commit_message>
Technical-verification corrections: D&A history, debt basis, GSK net-debt reconciliation, one-off revenue switch, DCF input validation, research v2.1 scope guard and set 4; home page lists completed simulations
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/pharma-valuation/pharma-valuation-model.xlsx
+++ b/public/downloads/pharma-valuation/pharma-valuation-model.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dave7\Desktop\CareerMaxing\website\public\downloads\pharma-valuation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCC415F7-A031-4BB3-95B6-003E60DBA6EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A32EF4AC-BDA7-48CA-A4F4-B3FCAC84EFBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5370" yWindow="915" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
     <t>Pharma Valuation Explorer: model workbook</t>
   </si>
   <si>
-    <t>Generated 2026-10-20 from public SEC XBRL data (Forms 20-F) and ECB reference rates.</t>
+    <t>Generated 2026-10-23 from public SEC XBRL data (Forms 20-F) and ECB reference rates.</t>
   </si>
   <si>
     <t>What this is</t>

</xml_diff>